<commit_message>
fix: preserve original video titles in download filenames
</commit_message>
<xml_diff>
--- a/docs/releases/StreamDrop-version-history.xlsx
+++ b/docs/releases/StreamDrop-version-history.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="1" r:id="R8c7bcb81ab8b450e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布明细" sheetId="2" r:id="R705f8557ee354035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="1" r:id="R3e3cbc1feeaa400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布明细" sheetId="2" r:id="Rb3ed9a71495243f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -557,36 +557,69 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="80" customHeight="1">
-      <x:c r="A10" s="11" t="str">
+      <x:c r="A10" s="8" t="str">
         <x:v>1.1.0</x:v>
       </x:c>
-      <x:c r="B10" s="12" t="d">
+      <x:c r="B10" s="9" t="d">
         <x:v>2026-10-18T12:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C10" s="11" t="str">
+      <x:c r="C10" s="8" t="str">
         <x:v>小版本</x:v>
       </x:c>
-      <x:c r="D10" s="11" t="str">
+      <x:c r="D10" s="8" t="str">
         <x:v>正式标签版本</x:v>
       </x:c>
-      <x:c r="E10" s="13" t="n">
+      <x:c r="E10" s="10" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F10" s="11" t="str">
+      <x:c r="F10" s="8" t="str">
         <x:v>v1.1.0</x:v>
       </x:c>
-      <x:c r="G10" s="11" t="str">
+      <x:c r="G10" s="8" t="str">
         <x:v>新增兼容的完成恢复与播放观察能力，旧数据可读。</x:v>
       </x:c>
-      <x:c r="H10" s="11" t="str">
+      <x:c r="H10" s="8" t="str">
         <x:v>统一终态与收尾；恢复完成提交；保存播放观察；建立 Excel 发布台账。</x:v>
       </x:c>
-      <x:c r="I10" s="13" t="n">
+      <x:c r="I10" s="10" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="J10" s="11" t="str">
+      <x:c r="J10" s="8" t="str">
         <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.0
 跨卷中断归属未知时保留现场；首帧不代表全片质量；未公证。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="80" customHeight="1">
+      <x:c r="A11" s="11" t="str">
+        <x:v>1.1.1</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="d">
+        <x:v>2026-10-19T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C11" s="11" t="str">
+        <x:v>补丁版本</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="str">
+        <x:v>正式标签版本</x:v>
+      </x:c>
+      <x:c r="E11" s="13" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F11" s="11" t="str">
+        <x:v>v1.1.1</x:v>
+      </x:c>
+      <x:c r="G11" s="11" t="str">
+        <x:v>修正下载文件名，保持旧数据和操作兼容。</x:v>
+      </x:c>
+      <x:c r="H11" s="11" t="str">
+        <x:v>保留中文和空格，移除自动追加的视频 ID；同名文件继续加编号防覆盖。</x:v>
+      </x:c>
+      <x:c r="I11" s="13" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="J11" s="11" t="str">
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.1
+仅对新下载生效；标题中的系统非法字符及长度仍需处理。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -614,7 +647,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>StreamDrop 1.1.0 发布明细</x:v>
+        <x:v>StreamDrop 1.1.1 发布明细</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -654,107 +687,56 @@
     </x:row>
     <x:row r="6" ht="68" customHeight="1">
       <x:c r="A6" s="8" t="str">
-        <x:v>下载执行</x:v>
+        <x:v>文件命名</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>统一停止意图、单次终态与资源收尾。</x:v>
+        <x:v>网页视频使用原始标题，不再强制 ASCII，也不自动追加方括号 ID。</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
-        <x:v>真实直链 15 轮暂停只结算一次，保留网页/HLS 回归。</x:v>
+        <x:v>真实 yt-dlp 下载含中文、空格和原有方括号的标题，两次下载验证同名不覆盖。</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>88941d449470150c67fbe211f6da90f6552a440f</x:v>
+        <x:v>v1.1.1</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/commit/88941d449470150c67fbe211f6da90f6552a440f</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="68" customHeight="1">
-      <x:c r="A7" s="8" t="str">
-        <x:v>完成提交</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="str">
-        <x:v>恢复落盘和保存中断，保留清理责任与用户删除选择。</x:v>
-      </x:c>
-      <x:c r="C7" s="8" t="str">
-        <x:v>连续保存失败、重载幂等、清理失败、外来目标保护。</x:v>
-      </x:c>
-      <x:c r="D7" s="8" t="str">
-        <x:v>9f84d695f7c6b6888d27a63d50bc90fbd60c0b1b</x:v>
-      </x:c>
-      <x:c r="E7" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/commit/9f84d695f7c6b6888d27a63d50bc90fbd60c0b1b</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="68" customHeight="1">
-      <x:c r="A8" s="8" t="str">
-        <x:v>播放观察</x:v>
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="2"/>
+      <x:c r="B7" s="2"/>
+      <x:c r="C7" s="2"/>
+      <x:c r="D7" s="2"/>
+      <x:c r="E7" s="2"/>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="14" t="str">
+        <x:v>兼容与限制</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>持久保存 decoded / converted / unknown / notChecked。</x:v>
-      </x:c>
-      <x:c r="C8" s="8" t="str">
-        <x:v>真实 VP9 转换、原生画面、未知原因及历史重载。</x:v>
-      </x:c>
-      <x:c r="D8" s="8" t="str">
-        <x:v>1df71629c452bf38b5b0856449566fdd4bdb419a</x:v>
-      </x:c>
-      <x:c r="E8" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/commit/1df71629c452bf38b5b0856449566fdd4bdb419a</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="68" customHeight="1">
-      <x:c r="A9" s="8" t="str">
-        <x:v>发布管理</x:v>
-      </x:c>
+        <x:v>旧数据可读；不回填旧记录的播放观察。</x:v>
+      </x:c>
+      <x:c r="C8" s="8"/>
+      <x:c r="D8" s="2"/>
+      <x:c r="E8" s="2"/>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="2"/>
       <x:c r="B9" s="8" t="str">
-        <x:v>统一版本来源、变更说明、Excel 台账与标签一致性检查。</x:v>
-      </x:c>
-      <x:c r="C9" s="8" t="str">
-        <x:v>检查 VERSION、构建号、所有 Excel 行、App 版本与 Git 标签。</x:v>
-      </x:c>
-      <x:c r="D9" s="8" t="str">
-        <x:v>v1.1.0</x:v>
-      </x:c>
-      <x:c r="E9" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
+        <x:v>跨卷中断无法确认身份时，保留现场并报告未知。</x:v>
+      </x:c>
+      <x:c r="C9" s="8"/>
+      <x:c r="D9" s="2"/>
+      <x:c r="E9" s="2"/>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="2"/>
-      <x:c r="B10" s="2"/>
-      <x:c r="C10" s="2"/>
+      <x:c r="B10" s="8" t="str">
+        <x:v>标签锚定最终提交；Excel 不写自身所属提交的 SHA。</x:v>
+      </x:c>
+      <x:c r="C10" s="8"/>
       <x:c r="D10" s="2"/>
       <x:c r="E10" s="2"/>
-    </x:row>
-    <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="14" t="str">
-        <x:v>兼容与限制</x:v>
-      </x:c>
-      <x:c r="B11" s="8" t="str">
-        <x:v>旧数据可读；不回填旧记录的播放观察。</x:v>
-      </x:c>
-      <x:c r="C11" s="8"/>
-      <x:c r="D11" s="2"/>
-      <x:c r="E11" s="2"/>
-    </x:row>
-    <x:row r="12" ht="42" customHeight="1">
-      <x:c r="A12" s="2"/>
-      <x:c r="B12" s="8" t="str">
-        <x:v>跨卷中断无法确认身份时，保留现场并报告未知。</x:v>
-      </x:c>
-      <x:c r="C12" s="8"/>
-      <x:c r="D12" s="2"/>
-      <x:c r="E12" s="2"/>
-    </x:row>
-    <x:row r="13" ht="42" customHeight="1">
-      <x:c r="A13" s="2"/>
-      <x:c r="B13" s="8" t="str">
-        <x:v>标签锚定最终提交；Excel 不写自身所属提交的 SHA。</x:v>
-      </x:c>
-      <x:c r="C13" s="8"/>
-      <x:c r="D13" s="2"/>
-      <x:c r="E13" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: release v1.1.2 with safe recovery and final filenames
</commit_message>
<xml_diff>
--- a/docs/releases/StreamDrop-version-history.xlsx
+++ b/docs/releases/StreamDrop-version-history.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="1" r:id="R3e3cbc1feeaa400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布明细" sheetId="2" r:id="Rb3ed9a71495243f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="1" r:id="Rc39636c9f53d4d32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布明细" sheetId="2" r:id="R0c67e2ae3cff421d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -590,36 +590,69 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="80" customHeight="1">
-      <x:c r="A11" s="11" t="str">
+      <x:c r="A11" s="8" t="str">
         <x:v>1.1.1</x:v>
       </x:c>
-      <x:c r="B11" s="12" t="d">
+      <x:c r="B11" s="9" t="d">
         <x:v>2026-10-19T12:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C11" s="11" t="str">
+      <x:c r="C11" s="8" t="str">
         <x:v>补丁版本</x:v>
       </x:c>
-      <x:c r="D11" s="11" t="str">
+      <x:c r="D11" s="8" t="str">
         <x:v>正式标签版本</x:v>
       </x:c>
-      <x:c r="E11" s="13" t="n">
+      <x:c r="E11" s="10" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="F11" s="11" t="str">
+      <x:c r="F11" s="8" t="str">
         <x:v>v1.1.1</x:v>
       </x:c>
-      <x:c r="G11" s="11" t="str">
+      <x:c r="G11" s="8" t="str">
         <x:v>修正下载文件名，保持旧数据和操作兼容。</x:v>
       </x:c>
-      <x:c r="H11" s="11" t="str">
+      <x:c r="H11" s="8" t="str">
         <x:v>保留中文和空格，移除自动追加的视频 ID；同名文件继续加编号防覆盖。</x:v>
       </x:c>
-      <x:c r="I11" s="13" t="n">
+      <x:c r="I11" s="10" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="J11" s="11" t="str">
+      <x:c r="J11" s="8" t="str">
         <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.1
 仅对新下载生效；标题中的系统非法字符及长度仍需处理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="80" customHeight="1">
+      <x:c r="A12" s="11" t="str">
+        <x:v>1.1.2</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="d">
+        <x:v>2026-10-20T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C12" s="11" t="str">
+        <x:v>补丁版本</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="str">
+        <x:v>正式标签版本</x:v>
+      </x:c>
+      <x:c r="E12" s="13" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F12" s="11" t="str">
+        <x:v>v1.1.2</x:v>
+      </x:c>
+      <x:c r="G12" s="11" t="str">
+        <x:v>修正既有存储恢复、长文件名和发布校验；旧数据可读，无需迁移。</x:v>
+      </x:c>
+      <x:c r="H12" s="11" t="str">
+        <x:v>统一写入许可；先恢复再重试；长标题保留扩展名与编号；发布说明统一来源。</x:v>
+      </x:c>
+      <x:c r="I12" s="13" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J12" s="11" t="str">
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.2
+未新测公共站点、跨卷中断、断电或 Intel/macOS 13 实机；未公证。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -647,7 +680,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>StreamDrop 1.1.1 发布明细</x:v>
+        <x:v>StreamDrop 1.1.2 发布明细</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -687,56 +720,99 @@
     </x:row>
     <x:row r="6" ht="68" customHeight="1">
       <x:c r="A6" s="8" t="str">
-        <x:v>文件命名</x:v>
+        <x:v>存储与完成恢复</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>网页视频使用原始标题，不再强制 ASCII，也不自动追加方括号 ID。</x:v>
+        <x:v>存储拥有写入许可；重试前恢复已有完成提交，清理最后才删除凭据。</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
-        <x:v>真实 yt-dlp 下载含中文、空格和原有方括号的标题，两次下载验证同名不覆盖。</x:v>
+        <x:v>损坏及未来状态拒绝各写入入口；无服务器时恢复成功；真实磁盘失败、清理及身份回归通过。</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>v1.1.1</x:v>
+        <x:v>v1.1.2</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="2"/>
-      <x:c r="B7" s="2"/>
-      <x:c r="C7" s="2"/>
-      <x:c r="D7" s="2"/>
-      <x:c r="E7" s="2"/>
-    </x:row>
-    <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="14" t="str">
-        <x:v>兼容与限制</x:v>
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="68" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>最终文件名</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>统一长度预算，先预留扩展名和同名编号，再缩短长标题。</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>长 ASCII、中文与复合 emoji 实际写入成功；扩展名保留、同名不覆盖；原网页标题测试通过。</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>v1.1.2</x:v>
+      </x:c>
+      <x:c r="E7" s="8" t="str">
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="68" customHeight="1">
+      <x:c r="A8" s="8" t="str">
+        <x:v>发布记录</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>旧数据可读；不回填旧记录的播放观察。</x:v>
-      </x:c>
-      <x:c r="C8" s="8"/>
-      <x:c r="D8" s="2"/>
-      <x:c r="E8" s="2"/>
-    </x:row>
-    <x:row r="9" ht="42" customHeight="1">
+        <x:v>发布校验使用显式错误；Excel 兼容说明来自发布数据并独立逐行校验。</x:v>
+      </x:c>
+      <x:c r="C8" s="8" t="str">
+        <x:v>3 项 Python 回归通过，均执行普通和 -O 模式；错误版本及说明漂移明确拒绝。</x:v>
+      </x:c>
+      <x:c r="D8" s="8" t="str">
+        <x:v>v1.1.2</x:v>
+      </x:c>
+      <x:c r="E8" s="8" t="str">
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
       <x:c r="A9" s="2"/>
-      <x:c r="B9" s="8" t="str">
-        <x:v>跨卷中断无法确认身份时，保留现场并报告未知。</x:v>
-      </x:c>
-      <x:c r="C9" s="8"/>
+      <x:c r="B9" s="2"/>
+      <x:c r="C9" s="2"/>
       <x:c r="D9" s="2"/>
       <x:c r="E9" s="2"/>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="2"/>
+      <x:c r="A10" s="14" t="str">
+        <x:v>兼容与限制</x:v>
+      </x:c>
       <x:c r="B10" s="8" t="str">
-        <x:v>标签锚定最终提交；Excel 不写自身所属提交的 SHA。</x:v>
+        <x:v>旧状态与旧完成凭据可读；损坏或未来版本状态保留并禁止写入。</x:v>
       </x:c>
       <x:c r="C10" s="8"/>
       <x:c r="D10" s="2"/>
       <x:c r="E10" s="2"/>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="2"/>
+      <x:c r="B11" s="8" t="str">
+        <x:v>长标题按保守 UTF-8 预算缩短，保留扩展名和同名编号；不重命名已有文件。</x:v>
+      </x:c>
+      <x:c r="C11" s="8"/>
+      <x:c r="D11" s="2"/>
+      <x:c r="E11" s="2"/>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="2"/>
+      <x:c r="B12" s="8" t="str">
+        <x:v>跨卷中断归属未知时保留现场；未验证断电及 Intel/macOS 13 实机。</x:v>
+      </x:c>
+      <x:c r="C12" s="8"/>
+      <x:c r="D12" s="2"/>
+      <x:c r="E12" s="2"/>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="2"/>
+      <x:c r="B13" s="8" t="str">
+        <x:v>标签锚定最终提交；Excel 不写自身所属提交的 SHA。</x:v>
+      </x:c>
+      <x:c r="C13" s="8"/>
+      <x:c r="D13" s="2"/>
+      <x:c r="E13" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: release v1.2.0 with graceful shutdown and tool diagnostics
</commit_message>
<xml_diff>
--- a/docs/releases/StreamDrop-version-history.xlsx
+++ b/docs/releases/StreamDrop-version-history.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="1" r:id="Rc39636c9f53d4d32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布明细" sheetId="2" r:id="R0c67e2ae3cff421d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="1" r:id="Rb5dd6b6eae6e427b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布明细" sheetId="2" r:id="Rf3dd507cd7b8482f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -623,36 +623,69 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="80" customHeight="1">
-      <x:c r="A12" s="11" t="str">
+      <x:c r="A12" s="8" t="str">
         <x:v>1.1.2</x:v>
       </x:c>
-      <x:c r="B12" s="12" t="d">
+      <x:c r="B12" s="9" t="d">
         <x:v>2026-10-20T12:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C12" s="11" t="str">
+      <x:c r="C12" s="8" t="str">
         <x:v>补丁版本</x:v>
       </x:c>
-      <x:c r="D12" s="11" t="str">
+      <x:c r="D12" s="8" t="str">
         <x:v>正式标签版本</x:v>
       </x:c>
-      <x:c r="E12" s="13" t="n">
+      <x:c r="E12" s="10" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="F12" s="11" t="str">
+      <x:c r="F12" s="8" t="str">
         <x:v>v1.1.2</x:v>
       </x:c>
-      <x:c r="G12" s="11" t="str">
+      <x:c r="G12" s="8" t="str">
         <x:v>修正既有存储恢复、长文件名和发布校验；旧数据可读，无需迁移。</x:v>
       </x:c>
-      <x:c r="H12" s="11" t="str">
+      <x:c r="H12" s="8" t="str">
         <x:v>统一写入许可；先恢复再重试；长标题保留扩展名与编号；发布说明统一来源。</x:v>
       </x:c>
-      <x:c r="I12" s="13" t="n">
+      <x:c r="I12" s="10" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="J12" s="11" t="str">
+      <x:c r="J12" s="8" t="str">
         <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.2
 未新测公共站点、跨卷中断、断电或 Intel/macOS 13 实机；未公证。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="80" customHeight="1">
+      <x:c r="A13" s="11" t="str">
+        <x:v>1.2.0</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="d">
+        <x:v>2026-10-20T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="str">
+        <x:v>小版本</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="str">
+        <x:v>正式标签版本</x:v>
+      </x:c>
+      <x:c r="E13" s="13" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F13" s="11" t="str">
+        <x:v>v1.2.0</x:v>
+      </x:c>
+      <x:c r="G13" s="11" t="str">
+        <x:v>新增兼容的工具运行检查和版本诊断能力，完善正常退出；旧数据无需迁移。</x:v>
+      </x:c>
+      <x:c r="H13" s="11" t="str">
+        <x:v>退出等待资源收尾；检查工具版本；复制完整诊断；CI 严格验证下载与发布记录。</x:v>
+      </x:c>
+      <x:c r="I13" s="13" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J13" s="11" t="str">
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.0
+强制退出及断电不保证正常收尾；未新测公共站点或 macOS 13 实机；未公证。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -680,7 +713,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>StreamDrop 1.1.2 发布明细</x:v>
+        <x:v>StreamDrop 1.2.0 发布明细</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -720,53 +753,53 @@
     </x:row>
     <x:row r="6" ht="68" customHeight="1">
       <x:c r="A6" s="8" t="str">
-        <x:v>存储与完成恢复</x:v>
+        <x:v>退出与完成恢复</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>存储拥有写入许可；重试前恢复已有完成提交，清理最后才删除凭据。</x:v>
+        <x:v>退出等待下载、转换和工具检查收尾；清理失败保留恢复凭据。</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
-        <x:v>损坏及未来状态拒绝各写入入口；无服务器时恢复成功；真实磁盘失败、清理及身份回归通过。</x:v>
+        <x:v>直链与转换阶段退出后重载完成且历史唯一；最终保存和凭据删除故障回归通过。</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>v1.1.2</x:v>
+        <x:v>v1.2.0</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.2</x:v>
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="68" customHeight="1">
       <x:c r="A7" s="8" t="str">
-        <x:v>最终文件名</x:v>
+        <x:v>工具与诊断</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
-        <x:v>统一长度预算，先预留扩展名和同名编号，再缩短长标题。</x:v>
+        <x:v>实际检查工具版本及运行状态，复制诊断附 App、系统和当前工具信息。</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
-        <x:v>长 ASCII、中文与复合 emoji 实际写入成功；扩展名保留、同名不覆盖；原网页标题测试通过。</x:v>
+        <x:v>真实工具检查、错误输出、缺失、失败、超时、取消及退出清理测试通过。</x:v>
       </x:c>
       <x:c r="D7" s="8" t="str">
-        <x:v>v1.1.2</x:v>
+        <x:v>v1.2.0</x:v>
       </x:c>
       <x:c r="E7" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.2</x:v>
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.0</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="68" customHeight="1">
       <x:c r="A8" s="8" t="str">
-        <x:v>发布记录</x:v>
+        <x:v>自动验证</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>发布校验使用显式错误；Excel 兼容说明来自发布数据并独立逐行校验。</x:v>
+        <x:v>GitHub macOS 工作流验证完整回归、版本 Excel、构建、签名及 DMG。</x:v>
       </x:c>
       <x:c r="C8" s="8" t="str">
-        <x:v>3 项 Python 回归通过，均执行普通和 -O 模式；错误版本及说明漂移明确拒绝。</x:v>
+        <x:v>严格模式拒绝缺工具、失败、跳过、空报告；实际 XCTest 跳过事件贯穿校验。</x:v>
       </x:c>
       <x:c r="D8" s="8" t="str">
-        <x:v>v1.1.2</x:v>
+        <x:v>v1.2.0</x:v>
       </x:c>
       <x:c r="E8" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.1.2</x:v>
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.0</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -781,7 +814,7 @@
         <x:v>兼容与限制</x:v>
       </x:c>
       <x:c r="B10" s="8" t="str">
-        <x:v>旧状态与旧完成凭据可读；损坏或未来版本状态保留并禁止写入。</x:v>
+        <x:v>旧偏好与下载历史可读，无需迁移；不修改已有下载文件。</x:v>
       </x:c>
       <x:c r="C10" s="8"/>
       <x:c r="D10" s="2"/>
@@ -790,7 +823,7 @@
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="2"/>
       <x:c r="B11" s="8" t="str">
-        <x:v>长标题按保守 UTF-8 预算缩短，保留扩展名和同名编号；不重命名已有文件。</x:v>
+        <x:v>正常退出等待资源结束；系统强制退出和断电不提供同等保证。</x:v>
       </x:c>
       <x:c r="C11" s="8"/>
       <x:c r="D11" s="2"/>
@@ -799,7 +832,7 @@
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="2"/>
       <x:c r="B12" s="8" t="str">
-        <x:v>跨卷中断归属未知时保留现场；未验证断电及 Intel/macOS 13 实机。</x:v>
+        <x:v>诊断中的工具版本在收集时检查，不代表失败发生时的版本。</x:v>
       </x:c>
       <x:c r="C12" s="8"/>
       <x:c r="D12" s="2"/>
@@ -808,11 +841,20 @@
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="2"/>
       <x:c r="B13" s="8" t="str">
-        <x:v>标签锚定最终提交；Excel 不写自身所属提交的 SHA。</x:v>
+        <x:v>本轮使用本地合成媒体；未重新验证公共站点或 macOS 13 实机。</x:v>
       </x:c>
       <x:c r="C13" s="8"/>
       <x:c r="D13" s="2"/>
       <x:c r="E13" s="2"/>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="2"/>
+      <x:c r="B14" s="8" t="str">
+        <x:v>跨卷中断归属未知时保留现场；App 为 ad-hoc 签名，未公证。</x:v>
+      </x:c>
+      <x:c r="C14" s="8"/>
+      <x:c r="D14" s="2"/>
+      <x:c r="E14" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: release v1.2.1 with bounded CI fixture startup
</commit_message>
<xml_diff>
--- a/docs/releases/StreamDrop-version-history.xlsx
+++ b/docs/releases/StreamDrop-version-history.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="1" r:id="Rb5dd6b6eae6e427b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布明细" sheetId="2" r:id="Rf3dd507cd7b8482f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="1" r:id="R9e2db75cea7e4c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布明细" sheetId="2" r:id="R30de9d71bd3e4dc8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -656,36 +656,69 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="80" customHeight="1">
-      <x:c r="A13" s="11" t="str">
+      <x:c r="A13" s="8" t="str">
         <x:v>1.2.0</x:v>
       </x:c>
-      <x:c r="B13" s="12" t="d">
+      <x:c r="B13" s="9" t="d">
         <x:v>2026-10-20T12:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C13" s="11" t="str">
+      <x:c r="C13" s="8" t="str">
         <x:v>小版本</x:v>
       </x:c>
-      <x:c r="D13" s="11" t="str">
+      <x:c r="D13" s="8" t="str">
         <x:v>正式标签版本</x:v>
       </x:c>
-      <x:c r="E13" s="13" t="n">
+      <x:c r="E13" s="10" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="F13" s="11" t="str">
+      <x:c r="F13" s="8" t="str">
         <x:v>v1.2.0</x:v>
       </x:c>
-      <x:c r="G13" s="11" t="str">
+      <x:c r="G13" s="8" t="str">
         <x:v>新增兼容的工具运行检查和版本诊断能力，完善正常退出；旧数据无需迁移。</x:v>
       </x:c>
-      <x:c r="H13" s="11" t="str">
+      <x:c r="H13" s="8" t="str">
         <x:v>退出等待资源收尾；检查工具版本；复制完整诊断；CI 严格验证下载与发布记录。</x:v>
       </x:c>
-      <x:c r="I13" s="13" t="n">
+      <x:c r="I13" s="10" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="J13" s="11" t="str">
+      <x:c r="J13" s="8" t="str">
         <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.0
 强制退出及断电不保证正常收尾；未新测公共站点或 macOS 13 实机；未公证。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="80" customHeight="1">
+      <x:c r="A14" s="11" t="str">
+        <x:v>1.2.1</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="d">
+        <x:v>2026-10-20T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C14" s="11" t="str">
+        <x:v>补丁版本</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="str">
+        <x:v>正式标签版本</x:v>
+      </x:c>
+      <x:c r="E14" s="13" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F14" s="11" t="str">
+        <x:v>v1.2.1</x:v>
+      </x:c>
+      <x:c r="G14" s="11" t="str">
+        <x:v>修正 CI 测试服务启动和诊断，不改变 App 操作或用户数据。</x:v>
+      </x:c>
+      <x:c r="H14" s="11" t="str">
+        <x:v>CI 使用系统 Python；就绪等待有界；记录实际启动耗时；服务退出立即失败。</x:v>
+      </x:c>
+      <x:c r="I14" s="13" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J14" s="11" t="str">
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.1
+1.2.0 首次 CI 启动失败的底层原因未确认；未扩大公共站点及硬件覆盖。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -713,7 +746,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>StreamDrop 1.2.0 发布明细</x:v>
+        <x:v>StreamDrop 1.2.1 发布明细</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -753,108 +786,56 @@
     </x:row>
     <x:row r="6" ht="68" customHeight="1">
       <x:c r="A6" s="8" t="str">
-        <x:v>退出与完成恢复</x:v>
+        <x:v>CI 启动与诊断</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>退出等待下载、转换和工具检查收尾；清理失败保留恢复凭据。</x:v>
+        <x:v>明确系统 Python，允许有界启动时间，记录就绪耗时并检查服务退出原因。</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
-        <x:v>直链与转换阶段退出后重载完成且历史唯一；最终保存和凭据删除故障回归通过。</x:v>
+        <x:v>真实退出码 7 的服务被立即拒绝；完整本地下载回归和发布门禁继续验证。</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>v1.2.0</x:v>
+        <x:v>v1.2.1</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="68" customHeight="1">
-      <x:c r="A7" s="8" t="str">
-        <x:v>工具与诊断</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="str">
-        <x:v>实际检查工具版本及运行状态，复制诊断附 App、系统和当前工具信息。</x:v>
-      </x:c>
-      <x:c r="C7" s="8" t="str">
-        <x:v>真实工具检查、错误输出、缺失、失败、超时、取消及退出清理测试通过。</x:v>
-      </x:c>
-      <x:c r="D7" s="8" t="str">
-        <x:v>v1.2.0</x:v>
-      </x:c>
-      <x:c r="E7" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="68" customHeight="1">
-      <x:c r="A8" s="8" t="str">
-        <x:v>自动验证</x:v>
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="2"/>
+      <x:c r="B7" s="2"/>
+      <x:c r="C7" s="2"/>
+      <x:c r="D7" s="2"/>
+      <x:c r="E7" s="2"/>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="14" t="str">
+        <x:v>兼容与限制</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>GitHub macOS 工作流验证完整回归、版本 Excel、构建、签名及 DMG。</x:v>
-      </x:c>
-      <x:c r="C8" s="8" t="str">
-        <x:v>严格模式拒绝缺工具、失败、跳过、空报告；实际 XCTest 跳过事件贯穿校验。</x:v>
-      </x:c>
-      <x:c r="D8" s="8" t="str">
-        <x:v>v1.2.0</x:v>
-      </x:c>
-      <x:c r="E8" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
+        <x:v>保持 1.2.0 的退出、工具检查与诊断功能，旧数据无需迁移。</x:v>
+      </x:c>
+      <x:c r="C8" s="8"/>
+      <x:c r="D8" s="2"/>
+      <x:c r="E8" s="2"/>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="2"/>
-      <x:c r="B9" s="2"/>
-      <x:c r="C9" s="2"/>
+      <x:c r="B9" s="8" t="str">
+        <x:v>CI 环境及测试启动修正；远端完整结果见 GitHub Release 链接。</x:v>
+      </x:c>
+      <x:c r="C9" s="8"/>
       <x:c r="D9" s="2"/>
       <x:c r="E9" s="2"/>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="14" t="str">
-        <x:v>兼容与限制</x:v>
-      </x:c>
+      <x:c r="A10" s="2"/>
       <x:c r="B10" s="8" t="str">
-        <x:v>旧偏好与下载历史可读，无需迁移；不修改已有下载文件。</x:v>
+        <x:v>不移动已发布标签；未新增公共站点、跨卷或 macOS 13 实机验证。</x:v>
       </x:c>
       <x:c r="C10" s="8"/>
       <x:c r="D10" s="2"/>
       <x:c r="E10" s="2"/>
-    </x:row>
-    <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="2"/>
-      <x:c r="B11" s="8" t="str">
-        <x:v>正常退出等待资源结束；系统强制退出和断电不提供同等保证。</x:v>
-      </x:c>
-      <x:c r="C11" s="8"/>
-      <x:c r="D11" s="2"/>
-      <x:c r="E11" s="2"/>
-    </x:row>
-    <x:row r="12" ht="42" customHeight="1">
-      <x:c r="A12" s="2"/>
-      <x:c r="B12" s="8" t="str">
-        <x:v>诊断中的工具版本在收集时检查，不代表失败发生时的版本。</x:v>
-      </x:c>
-      <x:c r="C12" s="8"/>
-      <x:c r="D12" s="2"/>
-      <x:c r="E12" s="2"/>
-    </x:row>
-    <x:row r="13" ht="42" customHeight="1">
-      <x:c r="A13" s="2"/>
-      <x:c r="B13" s="8" t="str">
-        <x:v>本轮使用本地合成媒体；未重新验证公共站点或 macOS 13 实机。</x:v>
-      </x:c>
-      <x:c r="C13" s="8"/>
-      <x:c r="D13" s="2"/>
-      <x:c r="E13" s="2"/>
-    </x:row>
-    <x:row r="14" ht="42" customHeight="1">
-      <x:c r="A14" s="2"/>
-      <x:c r="B14" s="8" t="str">
-        <x:v>跨卷中断归属未知时保留现场；App 为 ad-hoc 签名，未公证。</x:v>
-      </x:c>
-      <x:c r="C14" s="8"/>
-      <x:c r="D14" s="2"/>
-      <x:c r="E14" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: release v1.2.2 with a product-focused README and App copy
</commit_message>
<xml_diff>
--- a/docs/releases/StreamDrop-version-history.xlsx
+++ b/docs/releases/StreamDrop-version-history.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="1" r:id="R9e2db75cea7e4c5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布明细" sheetId="2" r:id="R30de9d71bd3e4dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本记录" sheetId="1" r:id="R0fea5971b1cf4b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布明细" sheetId="2" r:id="Re40a877427724ec9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -689,36 +689,69 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="80" customHeight="1">
-      <x:c r="A14" s="11" t="str">
+      <x:c r="A14" s="8" t="str">
         <x:v>1.2.1</x:v>
       </x:c>
-      <x:c r="B14" s="12" t="d">
+      <x:c r="B14" s="9" t="d">
         <x:v>2026-10-20T12:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C14" s="11" t="str">
+      <x:c r="C14" s="8" t="str">
         <x:v>补丁版本</x:v>
       </x:c>
-      <x:c r="D14" s="11" t="str">
+      <x:c r="D14" s="8" t="str">
         <x:v>正式标签版本</x:v>
       </x:c>
-      <x:c r="E14" s="13" t="n">
+      <x:c r="E14" s="10" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="F14" s="11" t="str">
+      <x:c r="F14" s="8" t="str">
         <x:v>v1.2.1</x:v>
       </x:c>
-      <x:c r="G14" s="11" t="str">
+      <x:c r="G14" s="8" t="str">
         <x:v>修正 CI 测试服务启动和诊断，不改变 App 操作或用户数据。</x:v>
       </x:c>
-      <x:c r="H14" s="11" t="str">
+      <x:c r="H14" s="8" t="str">
         <x:v>CI 使用系统 Python；就绪等待有界；记录实际启动耗时；服务退出立即失败。</x:v>
       </x:c>
-      <x:c r="I14" s="13" t="n">
+      <x:c r="I14" s="10" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="J14" s="11" t="str">
+      <x:c r="J14" s="8" t="str">
         <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.1
 1.2.0 首次 CI 启动失败的底层原因未确认；未扩大公共站点及硬件覆盖。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="80" customHeight="1">
+      <x:c r="A15" s="11" t="str">
+        <x:v>1.2.2</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="d">
+        <x:v>2026-10-20T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C15" s="11" t="str">
+        <x:v>补丁版本</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="str">
+        <x:v>正式标签版本</x:v>
+      </x:c>
+      <x:c r="E15" s="13" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F15" s="11" t="str">
+        <x:v>v1.2.2</x:v>
+      </x:c>
+      <x:c r="G15" s="11" t="str">
+        <x:v>仅修改项目介绍与 App 文案，下载行为和旧数据保持兼容。</x:v>
+      </x:c>
+      <x:c r="H15" s="11" t="str">
+        <x:v>重写 README，移除 App 内多余的第三方关系说明，同步 GitHub 首页介绍。</x:v>
+      </x:c>
+      <x:c r="I15" s="13" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="J15" s="11" t="str">
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.2
+40 项下载回归为前版通过基线，本版文案变更以构建及界面核对验证；未新增站点覆盖。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -746,7 +779,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>StreamDrop 1.2.1 发布明细</x:v>
+        <x:v>StreamDrop 1.2.2 发布明细</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -786,43 +819,51 @@
     </x:row>
     <x:row r="6" ht="68" customHeight="1">
       <x:c r="A6" s="8" t="str">
-        <x:v>CI 启动与诊断</x:v>
+        <x:v>项目介绍</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>明确系统 Python，允许有界启动时间，记录就绪耗时并检查服务退出原因。</x:v>
+        <x:v>从项目用途、功能、安装、工具依赖、快捷键和数据方式介绍 StreamDrop。</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
-        <x:v>真实退出码 7 的服务被立即拒绝；完整本地下载回归和发布门禁继续验证。</x:v>
+        <x:v>核对功能与源码一致，GitHub 默认分支 README 与发布版正文保持一致。</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>v1.2.1</x:v>
+        <x:v>v1.2.2</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
-        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="2"/>
-      <x:c r="B7" s="2"/>
-      <x:c r="C7" s="2"/>
-      <x:c r="D7" s="2"/>
-      <x:c r="E7" s="2"/>
-    </x:row>
-    <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="14" t="str">
-        <x:v>兼容与限制</x:v>
-      </x:c>
-      <x:c r="B8" s="8" t="str">
-        <x:v>保持 1.2.0 的退出、工具检查与诊断功能，旧数据无需迁移。</x:v>
-      </x:c>
-      <x:c r="C8" s="8"/>
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="68" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>App 文案</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>关于、使用说明、隐私和打包信息直接介绍产品，不再强调第三方关系。</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>源码及打包文档搜索无相关措辞，构建与安装后界面核对。</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>v1.2.2</x:v>
+      </x:c>
+      <x:c r="E7" s="8" t="str">
+        <x:v>https://github.com/profundity-max/StreamDrop/releases/tag/v1.2.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="2"/>
+      <x:c r="B8" s="2"/>
+      <x:c r="C8" s="2"/>
       <x:c r="D8" s="2"/>
       <x:c r="E8" s="2"/>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="2"/>
+      <x:c r="A9" s="14" t="str">
+        <x:v>兼容与限制</x:v>
+      </x:c>
       <x:c r="B9" s="8" t="str">
-        <x:v>CI 环境及测试启动修正；远端完整结果见 GitHub Release 链接。</x:v>
+        <x:v>文档与界面文案更新，不改变下载流程、偏好和本地历史。</x:v>
       </x:c>
       <x:c r="C9" s="8"/>
       <x:c r="D9" s="2"/>
@@ -831,11 +872,20 @@
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="2"/>
       <x:c r="B10" s="8" t="str">
-        <x:v>不移动已发布标签；未新增公共站点、跨卷或 macOS 13 实机验证。</x:v>
+        <x:v>测试数沿用 1.2.1 的 40 项基线；本版执行发布门禁、构建和界面核对。</x:v>
       </x:c>
       <x:c r="C10" s="8"/>
       <x:c r="D10" s="2"/>
       <x:c r="E10" s="2"/>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="2"/>
+      <x:c r="B11" s="8" t="str">
+        <x:v>默认分支同步 README；当前实现仍位于开发分支与发布标签。</x:v>
+      </x:c>
+      <x:c r="C11" s="8"/>
+      <x:c r="D11" s="2"/>
+      <x:c r="E11" s="2"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>